<commit_message>
Updated SRB_grids_kan model - 2026-08-26 12:05
</commit_message>
<xml_diff>
--- a/VerveStacks_IND_grids_kan10/SysSettings.xlsx
+++ b/VerveStacks_IND_grids_kan10/SysSettings.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\VEDA\Veda\Veda_models\vervestacks_models\VerveStacks_IND_grids_kan10\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FE754BB-D272-42A0-88D7-4A1140300A3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C913182-F64E-49ED-81A4-F8F0C953F6A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2340" windowWidth="28935" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="system_settings" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2061" uniqueCount="648">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2063" uniqueCount="650">
   <si>
     <t>~BookRegions_Map</t>
   </si>
@@ -1984,6 +1984,12 @@
   </si>
   <si>
     <t>heat at grid node -- way/201845280-765 (Wardha, 14 km)</t>
+  </si>
+  <si>
+    <t>UP,LO</t>
+  </si>
+  <si>
+    <t>act_bnd</t>
   </si>
 </sst>
 </file>
@@ -9937,7 +9943,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A64C410-895F-4040-A7AB-3F7211AA7FBD}">
-  <dimension ref="B1:N42"/>
+  <dimension ref="B1:N43"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12"/>
   <cols>
     <col min="1" max="1" width="11.42578125" style="11"/>
@@ -10090,49 +10096,52 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="2:12">
-      <c r="B14" s="14" t="s">
+    <row r="12" spans="2:12">
+      <c r="C12" s="11" t="s">
+        <v>648</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>649</v>
+      </c>
+      <c r="E12" s="11">
+        <v>0</v>
+      </c>
+      <c r="F12" s="11">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="2:12">
+      <c r="B15" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="G14" s="14"/>
-      <c r="H14" s="14"/>
-      <c r="I14" s="14"/>
-    </row>
-    <row r="15" spans="2:12">
-      <c r="B15" s="15" t="s">
+      <c r="G15" s="14"/>
+      <c r="H15" s="14"/>
+      <c r="I15" s="14"/>
+    </row>
+    <row r="16" spans="2:12">
+      <c r="B16" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="C15" s="15" t="s">
+      <c r="C16" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="D15" s="15" t="s">
+      <c r="D16" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="E15" s="15" t="s">
+      <c r="E16" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="F15" s="15" t="s">
+      <c r="F16" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="G15" s="15" t="s">
+      <c r="G16" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="H15" s="15" t="s">
+      <c r="H16" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="I15" s="15" t="s">
+      <c r="I16" s="15" t="s">
         <v>56</v>
-      </c>
-    </row>
-    <row r="16" spans="2:12">
-      <c r="D16" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="F16" s="11">
-        <v>2222</v>
-      </c>
-      <c r="G16" s="11" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="17" spans="2:14">
@@ -10140,35 +10149,35 @@
         <v>66</v>
       </c>
       <c r="F17" s="11">
-        <v>8888</v>
+        <v>2222</v>
       </c>
       <c r="G17" s="11" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="18" spans="2:14" ht="12.75">
-      <c r="B18" s="13"/>
-      <c r="C18" s="13"/>
+        <v>67</v>
+      </c>
+    </row>
+    <row r="18" spans="2:14">
       <c r="D18" s="11" t="s">
-        <v>236</v>
+        <v>66</v>
       </c>
       <c r="F18" s="11">
         <v>8888</v>
       </c>
       <c r="G18" s="11" t="s">
-        <v>235</v>
-      </c>
-      <c r="H18" s="13"/>
-      <c r="I18" s="13"/>
-      <c r="J18" s="13"/>
+        <v>234</v>
+      </c>
     </row>
     <row r="19" spans="2:14" ht="12.75">
       <c r="B19" s="13"/>
       <c r="C19" s="13"/>
-      <c r="D19" s="13"/>
-      <c r="E19" s="13"/>
-      <c r="F19" s="13"/>
-      <c r="G19" s="13"/>
+      <c r="D19" s="11" t="s">
+        <v>236</v>
+      </c>
+      <c r="F19" s="11">
+        <v>8888</v>
+      </c>
+      <c r="G19" s="11" t="s">
+        <v>235</v>
+      </c>
       <c r="H19" s="13"/>
       <c r="I19" s="13"/>
       <c r="J19" s="13"/>
@@ -10184,20 +10193,16 @@
       <c r="I20" s="13"/>
       <c r="J20" s="13"/>
     </row>
-    <row r="21" spans="2:14" ht="15">
-      <c r="B21"/>
-      <c r="C21"/>
-      <c r="D21"/>
-      <c r="E21"/>
-      <c r="F21"/>
-      <c r="G21"/>
-      <c r="H21"/>
-      <c r="I21"/>
-      <c r="J21"/>
-      <c r="K21"/>
-      <c r="L21"/>
-      <c r="M21"/>
-      <c r="N21"/>
+    <row r="21" spans="2:14" ht="12.75">
+      <c r="B21" s="13"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="13"/>
+      <c r="F21" s="13"/>
+      <c r="G21" s="13"/>
+      <c r="H21" s="13"/>
+      <c r="I21" s="13"/>
+      <c r="J21" s="13"/>
     </row>
     <row r="22" spans="2:14" ht="15">
       <c r="B22"/>
@@ -10513,6 +10518,21 @@
       <c r="L42"/>
       <c r="M42"/>
       <c r="N42"/>
+    </row>
+    <row r="43" spans="2:14" ht="15">
+      <c r="B43"/>
+      <c r="C43"/>
+      <c r="D43"/>
+      <c r="E43"/>
+      <c r="F43"/>
+      <c r="G43"/>
+      <c r="H43"/>
+      <c r="I43"/>
+      <c r="J43"/>
+      <c r="K43"/>
+      <c r="L43"/>
+      <c r="M43"/>
+      <c r="N43"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>